<commit_message>
feat: add English (/en/) versions of HBM and news-article pages
Locale-aware nav/footer/sub-nav fragments and load-more label so /en/
pages render English chrome while /kr/ pages are unchanged. Adds English
nav/footer fragments, EN import scripts, and imported EN content reports.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-hbm-overview.report.xlsx
+++ b/tools/importer/reports/import-hbm-overview.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="73">
   <si>
     <t>_reportFile</t>
   </si>
@@ -37,28 +37,199 @@
     <t>url</t>
   </si>
   <si>
+    <t>en/dram/hbm.report.json</t>
+  </si>
+  <si>
+    <t>["hero-product","columns-spec","columns-spec","columns-spec","accordion-faq","cards-content","cards-content"]</t>
+  </si>
+  <si>
+    <t>en/dram/hbm</t>
+  </si>
+  <si>
+    <t>success</t>
+  </si>
+  <si>
+    <t>hbm-overview</t>
+  </si>
+  <si>
+    <t>2026-06-29T03:27:12.549Z</t>
+  </si>
+  <si>
+    <t>HBM | DRAM | Samsung Semiconductor Global</t>
+  </si>
+  <si>
+    <t>https://semiconductor.samsung.com/us/dram/hbm/</t>
+  </si>
+  <si>
     <t>kr/dram/hbm.report.json</t>
   </si>
   <si>
-    <t>["hero-product","columns-spec","columns-spec","columns-spec","accordion-faq","cards-content","cards-content"]</t>
-  </si>
-  <si>
     <t>kr/dram/hbm</t>
   </si>
   <si>
-    <t>success</t>
-  </si>
-  <si>
-    <t>hbm-overview</t>
-  </si>
-  <si>
-    <t>2026-06-28T16:05:08.288Z</t>
+    <t>2026-06-29T03:27:32.939Z</t>
   </si>
   <si>
     <t>HBM | DRAM | 삼성반도체</t>
   </si>
   <si>
     <t>https://semiconductor.samsung.com/kr/dram/hbm/</t>
+  </si>
+  <si>
+    <t>en/news-events/news/samsung-electronics-begins-shipment-of-industry-first-hbm4e-samples.report.json</t>
+  </si>
+  <si>
+    <t>["article-header","tags-hashtag","tags-hashtag","banner-newsroom","cards-news"]</t>
+  </si>
+  <si>
+    <t>en/news-events/news/samsung-electronics-begins-shipment-of-industry-first-hbm4e-samples</t>
+  </si>
+  <si>
+    <t>news-article</t>
+  </si>
+  <si>
+    <t>2026-06-29T03:21:55.475Z</t>
+  </si>
+  <si>
+    <t>Samsung Electronics Begins Shipment of Industry-First HBM4E Samples | Samsung Semiconductor Global</t>
+  </si>
+  <si>
+    <t>https://semiconductor.samsung.com/us/news-events/news/samsung-electronics-begins-shipment-of-industry-first-hbm4e-samples/</t>
+  </si>
+  <si>
+    <t>en/news-events/news/samsung-ships-industry-first-commercial-hbm4-with-ultimate-performance-for-ai-computing.report.json</t>
+  </si>
+  <si>
+    <t>en/news-events/news/samsung-ships-industry-first-commercial-hbm4-with-ultimate-performance-for-ai-computing</t>
+  </si>
+  <si>
+    <t>2026-06-29T03:22:04.355Z</t>
+  </si>
+  <si>
+    <t>Samsung Ships Industry-First Commercial HBM4 With Ultimate Performance for AI Computing | Samsung Semiconductor Global</t>
+  </si>
+  <si>
+    <t>https://semiconductor.samsung.com/us/news-events/news/samsung-ships-industry-first-commercial-hbm4-with-ultimate-performance-for-ai-computing/</t>
+  </si>
+  <si>
+    <t>en/news-events/tech-blog/a-peek-into-ssd-virtualization.report.json</t>
+  </si>
+  <si>
+    <t>["article-header","article-image","tags-hashtag","tags-hashtag","cards-news"]</t>
+  </si>
+  <si>
+    <t>en/news-events/tech-blog/a-peek-into-ssd-virtualization</t>
+  </si>
+  <si>
+    <t>2026-06-29T03:22:57.039Z</t>
+  </si>
+  <si>
+    <t>A Peek into SSD Virtualization | Samsung Semiconductor Global</t>
+  </si>
+  <si>
+    <t>https://semiconductor.samsung.com/us/news-events/tech-blog/a-peek-into-ssd-virtualization/</t>
+  </si>
+  <si>
+    <t>en/us/dram/hbm.report.json</t>
+  </si>
+  <si>
+    <t>en/us/dram/hbm</t>
+  </si>
+  <si>
+    <t>2026-06-29T03:19:46.780Z</t>
+  </si>
+  <si>
+    <t>kr/news-events/news/samsung-electronics-begins-shipment-of-industry-first-hbm4e-samples.report.json</t>
+  </si>
+  <si>
+    <t>["article-header","article-image","article-image","tags-hashtag","tags-hashtag","banner-newsroom","cards-news"]</t>
+  </si>
+  <si>
+    <t>kr/news-events/news/samsung-electronics-begins-shipment-of-industry-first-hbm4e-samples</t>
+  </si>
+  <si>
+    <t>2026-06-29T02:50:23.205Z</t>
+  </si>
+  <si>
+    <t>삼성전자, 세계 최초 HBM4E 12단 샘플 출하 | 삼성반도체</t>
+  </si>
+  <si>
+    <t>https://semiconductor.samsung.com/kr/news-events/news/samsung-electronics-begins-shipment-of-industry-first-hbm4e-samples/</t>
+  </si>
+  <si>
+    <t>kr/news-events/news/samsung-ships-industry-first-commercial-hbm4-with-ultimate-performance-for-ai-computing.report.json</t>
+  </si>
+  <si>
+    <t>kr/news-events/news/samsung-ships-industry-first-commercial-hbm4-with-ultimate-performance-for-ai-computing</t>
+  </si>
+  <si>
+    <t>2026-06-29T02:50:31.855Z</t>
+  </si>
+  <si>
+    <t>삼성전자, 세계 최초 업계 최고 성능의 HBM4 양산 출하 | 삼성반도체</t>
+  </si>
+  <si>
+    <t>https://semiconductor.samsung.com/kr/news-events/news/samsung-ships-industry-first-commercial-hbm4-with-ultimate-performance-for-ai-computing/</t>
+  </si>
+  <si>
+    <t>kr/news-events/tech-blog/a-peek-into-ssd-virtualization.report.json</t>
+  </si>
+  <si>
+    <t>kr/news-events/tech-blog/a-peek-into-ssd-virtualization</t>
+  </si>
+  <si>
+    <t>2026-06-29T02:49:35.717Z</t>
+  </si>
+  <si>
+    <t>SSD 가상화 기술이 바꾸는 차세대 시스템 아키텍처 | 삼성반도체</t>
+  </si>
+  <si>
+    <t>https://semiconductor.samsung.com/kr/news-events/tech-blog/a-peek-into-ssd-virtualization/</t>
+  </si>
+  <si>
+    <t>kr/news-events/tech-blog/samsung-showcases-next-generationa-ai-semiconductor-innovations-at-computex-2026.report.json</t>
+  </si>
+  <si>
+    <t>["article-header","article-image","article-image","article-image","tags-hashtag","tags-hashtag","cards-news"]</t>
+  </si>
+  <si>
+    <t>kr/news-events/tech-blog/samsung-showcases-next-generationa-ai-semiconductor-innovations-at-computex-2026</t>
+  </si>
+  <si>
+    <t>2026-06-29T02:52:21.869Z</t>
+  </si>
+  <si>
+    <t>삼성전자, COMPUTEX 2026에서 AI 시대 반도체 경쟁력의 새로운 기준을 제시하다. | 삼성반도체</t>
+  </si>
+  <si>
+    <t>https://semiconductor.samsung.com/kr/news-events/tech-blog/samsung-showcases-next-generationa-ai-semiconductor-innovations-at-computex-2026/</t>
+  </si>
+  <si>
+    <t>en/us/news-events/news/samsung-electronics-begins-shipment-of-industry-first-hbm4e-samples.report.json</t>
+  </si>
+  <si>
+    <t>en/us/news-events/news/samsung-electronics-begins-shipment-of-industry-first-hbm4e-samples</t>
+  </si>
+  <si>
+    <t>2026-06-29T03:20:24.111Z</t>
+  </si>
+  <si>
+    <t>en/us/news-events/news/samsung-ships-industry-first-commercial-hbm4-with-ultimate-performance-for-ai-computing.report.json</t>
+  </si>
+  <si>
+    <t>en/us/news-events/news/samsung-ships-industry-first-commercial-hbm4-with-ultimate-performance-for-ai-computing</t>
+  </si>
+  <si>
+    <t>2026-06-29T03:20:31.204Z</t>
+  </si>
+  <si>
+    <t>en/us/news-events/tech-blog/a-peek-into-ssd-virtualization.report.json</t>
+  </si>
+  <si>
+    <t>en/us/news-events/tech-blog/a-peek-into-ssd-virtualization</t>
+  </si>
+  <si>
+    <t>2026-06-29T03:20:38.928Z</t>
   </si>
 </sst>
 </file>
@@ -447,16 +618,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H14"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="25" customWidth="1"/>
-    <col min="2" max="2" width="50" customWidth="1"/>
-    <col min="3" max="3" width="13" customWidth="1"/>
+    <col min="1" max="3" width="50" customWidth="1"/>
     <col min="5" max="5" width="14" customWidth="1"/>
     <col min="6" max="6" width="26" customWidth="1"/>
-    <col min="7" max="7" width="20" customWidth="1"/>
-    <col min="8" max="8" width="48" customWidth="1"/>
+    <col min="7" max="8" width="50" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.25">
@@ -509,6 +677,318 @@
       </c>
       <c r="H2" t="s">
         <v>15</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3" t="s">
+        <v>17</v>
+      </c>
+      <c r="D3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F3" t="s">
+        <v>18</v>
+      </c>
+      <c r="G3" t="s">
+        <v>19</v>
+      </c>
+      <c r="H3" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>21</v>
+      </c>
+      <c r="B4" t="s">
+        <v>22</v>
+      </c>
+      <c r="C4" t="s">
+        <v>23</v>
+      </c>
+      <c r="D4" t="s">
+        <v>11</v>
+      </c>
+      <c r="E4" t="s">
+        <v>24</v>
+      </c>
+      <c r="F4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G4" t="s">
+        <v>26</v>
+      </c>
+      <c r="H4" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>28</v>
+      </c>
+      <c r="B5" t="s">
+        <v>22</v>
+      </c>
+      <c r="C5" t="s">
+        <v>29</v>
+      </c>
+      <c r="D5" t="s">
+        <v>11</v>
+      </c>
+      <c r="E5" t="s">
+        <v>24</v>
+      </c>
+      <c r="F5" t="s">
+        <v>30</v>
+      </c>
+      <c r="G5" t="s">
+        <v>31</v>
+      </c>
+      <c r="H5" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>33</v>
+      </c>
+      <c r="B6" t="s">
+        <v>34</v>
+      </c>
+      <c r="C6" t="s">
+        <v>35</v>
+      </c>
+      <c r="D6" t="s">
+        <v>11</v>
+      </c>
+      <c r="E6" t="s">
+        <v>24</v>
+      </c>
+      <c r="F6" t="s">
+        <v>36</v>
+      </c>
+      <c r="G6" t="s">
+        <v>37</v>
+      </c>
+      <c r="H6" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>39</v>
+      </c>
+      <c r="B7" t="s">
+        <v>9</v>
+      </c>
+      <c r="C7" t="s">
+        <v>40</v>
+      </c>
+      <c r="D7" t="s">
+        <v>11</v>
+      </c>
+      <c r="E7" t="s">
+        <v>12</v>
+      </c>
+      <c r="F7" t="s">
+        <v>41</v>
+      </c>
+      <c r="G7" t="s">
+        <v>14</v>
+      </c>
+      <c r="H7" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>42</v>
+      </c>
+      <c r="B8" t="s">
+        <v>43</v>
+      </c>
+      <c r="C8" t="s">
+        <v>44</v>
+      </c>
+      <c r="D8" t="s">
+        <v>11</v>
+      </c>
+      <c r="E8" t="s">
+        <v>24</v>
+      </c>
+      <c r="F8" t="s">
+        <v>45</v>
+      </c>
+      <c r="G8" t="s">
+        <v>46</v>
+      </c>
+      <c r="H8" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>48</v>
+      </c>
+      <c r="B9" t="s">
+        <v>43</v>
+      </c>
+      <c r="C9" t="s">
+        <v>49</v>
+      </c>
+      <c r="D9" t="s">
+        <v>11</v>
+      </c>
+      <c r="E9" t="s">
+        <v>24</v>
+      </c>
+      <c r="F9" t="s">
+        <v>50</v>
+      </c>
+      <c r="G9" t="s">
+        <v>51</v>
+      </c>
+      <c r="H9" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>53</v>
+      </c>
+      <c r="B10" t="s">
+        <v>34</v>
+      </c>
+      <c r="C10" t="s">
+        <v>54</v>
+      </c>
+      <c r="D10" t="s">
+        <v>11</v>
+      </c>
+      <c r="E10" t="s">
+        <v>24</v>
+      </c>
+      <c r="F10" t="s">
+        <v>55</v>
+      </c>
+      <c r="G10" t="s">
+        <v>56</v>
+      </c>
+      <c r="H10" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>58</v>
+      </c>
+      <c r="B11" t="s">
+        <v>59</v>
+      </c>
+      <c r="C11" t="s">
+        <v>60</v>
+      </c>
+      <c r="D11" t="s">
+        <v>11</v>
+      </c>
+      <c r="E11" t="s">
+        <v>24</v>
+      </c>
+      <c r="F11" t="s">
+        <v>61</v>
+      </c>
+      <c r="G11" t="s">
+        <v>62</v>
+      </c>
+      <c r="H11" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>64</v>
+      </c>
+      <c r="B12" t="s">
+        <v>22</v>
+      </c>
+      <c r="C12" t="s">
+        <v>65</v>
+      </c>
+      <c r="D12" t="s">
+        <v>11</v>
+      </c>
+      <c r="E12" t="s">
+        <v>24</v>
+      </c>
+      <c r="F12" t="s">
+        <v>66</v>
+      </c>
+      <c r="G12" t="s">
+        <v>26</v>
+      </c>
+      <c r="H12" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>67</v>
+      </c>
+      <c r="B13" t="s">
+        <v>22</v>
+      </c>
+      <c r="C13" t="s">
+        <v>68</v>
+      </c>
+      <c r="D13" t="s">
+        <v>11</v>
+      </c>
+      <c r="E13" t="s">
+        <v>24</v>
+      </c>
+      <c r="F13" t="s">
+        <v>69</v>
+      </c>
+      <c r="G13" t="s">
+        <v>31</v>
+      </c>
+      <c r="H13" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>70</v>
+      </c>
+      <c r="B14" t="s">
+        <v>34</v>
+      </c>
+      <c r="C14" t="s">
+        <v>71</v>
+      </c>
+      <c r="D14" t="s">
+        <v>11</v>
+      </c>
+      <c r="E14" t="s">
+        <v>24</v>
+      </c>
+      <c r="F14" t="s">
+        <v>72</v>
+      </c>
+      <c r="G14" t="s">
+        <v>37</v>
+      </c>
+      <c r="H14" t="s">
+        <v>38</v>
       </c>
     </row>
   </sheetData>

</xml_diff>